<commit_message>
Freeze first column in weekly report template
</commit_message>
<xml_diff>
--- a/AIR_Weekly_Report_Template_June2026.xlsx
+++ b/AIR_Weekly_Report_Template_June2026.xlsx
@@ -83,7 +83,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -105,11 +105,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -135,6 +179,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2484,6 +2530,13 @@
         </is>
       </c>
       <c r="B90" s="6" t="n"/>
+      <c r="C90" s="9" t="n"/>
+      <c r="D90" s="9" t="n"/>
+      <c r="E90" s="9" t="n"/>
+      <c r="F90" s="9" t="n"/>
+      <c r="G90" s="9" t="n"/>
+      <c r="H90" s="9" t="n"/>
+      <c r="I90" s="10" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
@@ -2492,6 +2545,13 @@
         </is>
       </c>
       <c r="B92" s="6" t="n"/>
+      <c r="C92" s="9" t="n"/>
+      <c r="D92" s="9" t="n"/>
+      <c r="E92" s="9" t="n"/>
+      <c r="F92" s="9" t="n"/>
+      <c r="G92" s="9" t="n"/>
+      <c r="H92" s="9" t="n"/>
+      <c r="I92" s="10" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
@@ -2500,14 +2560,21 @@
         </is>
       </c>
       <c r="B94" s="6" t="n"/>
+      <c r="C94" s="9" t="n"/>
+      <c r="D94" s="9" t="n"/>
+      <c r="E94" s="9" t="n"/>
+      <c r="F94" s="9" t="n"/>
+      <c r="G94" s="9" t="n"/>
+      <c r="H94" s="9" t="n"/>
+      <c r="I94" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B92:I92"/>
+    <mergeCell ref="A57:I57"/>
     <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A76:I76"/>
     <mergeCell ref="A89:I89"/>

</xml_diff>